<commit_message>
audit(2026-06-17): record PR #211 in PRs-opened sheet
</commit_message>
<xml_diff>
--- a/audits/daily_usability_audit_2026-06-17.xlsx
+++ b/audits/daily_usability_audit_2026-06-17.xlsx
@@ -11190,7 +11190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11326,6 +11326,38 @@
       <c r="F4" s="9" t="inlineStr">
         <is>
           <t>All standard + light-mode + regression tests PASS today. New today: commit 093f5d0 / PR #210 'security(edge): rate-limit public endpoints + CRON_SECRET for scheduler functions' landed at 08:01 PT - 5 edge functions now per-IP rate-limited (60/min). 2 Instrumentl gap items (FM-IC-CFG-001 custom fields FAIL Low, FM-IC-CFG-002 public API PARTIAL Low) deferred to fundermatch-feature-builder task per spec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>SpikeyCoder/funder-finder</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>audit/2026-06-17</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>audit(2026-06-17): daily usability audit report</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>https://github.com/SpikeyCoder/funder-finder/pull/211</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Audit deliverable PR. Carries today's daily_usability_audit_2026-06-17.xlsx + build_audit_xlsx_2026-06-17.py. No code-fix PRs needed — all standard 8-category audits + light mode + regressions PASS.</t>
         </is>
       </c>
     </row>

</xml_diff>